<commit_message>
Unify contact settlement order and add timed resource drops with configured combat rules
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/battle_geometry.xlsx
+++ b/space-battleship/config_excel/battle_geometry.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="battle_geometry" sheetId="1" r:id="Re1dcba95695d4b8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="battle_geometry" sheetId="1" r:id="R067f9d3e22754e97"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -604,6 +604,61 @@
         <x:v>原固定舰体尺寸算法四艘起的宽度上限</x:v>
       </x:c>
     </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="1" t="str">
+        <x:v>projectile_min_x</x:v>
+      </x:c>
+      <x:c r="B31" s="1" t="n">
+        <x:v>-32</x:v>
+      </x:c>
+      <x:c r="C31" s="1" t="str">
+        <x:v>Existing native projectile retirement: left logical boundary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="1" t="str">
+        <x:v>projectile_max_x</x:v>
+      </x:c>
+      <x:c r="B32" s="1" t="n">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c r="C32" s="1" t="str">
+        <x:v>Existing native projectile retirement: right logical boundary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="1" t="str">
+        <x:v>projectile_min_y</x:v>
+      </x:c>
+      <x:c r="B33" s="1" t="n">
+        <x:v>-32</x:v>
+      </x:c>
+      <x:c r="C33" s="1" t="str">
+        <x:v>Existing native projectile retirement: upper logical boundary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="1" t="str">
+        <x:v>projectile_max_y</x:v>
+      </x:c>
+      <x:c r="B34" s="1" t="n">
+        <x:v>776</x:v>
+      </x:c>
+      <x:c r="C34" s="1" t="str">
+        <x:v>Existing native projectile retirement: lower logical boundary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="1" t="str">
+        <x:v>timed_drop_spawn_y</x:v>
+      </x:c>
+      <x:c r="B35" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C35" s="1" t="str">
+        <x:v>Design 01: timed resources enter from the top; X uses player_x.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>